<commit_message>
Banco de preguntas en Excel de ida y vuelta
El administrador descarga la plantilla vacía o el banco actual, lo edita y lo
vuelve a subir en /admin/preguntas:

- fila sin id: pregunta nueva, como borrador;
- fila con id y cambios: versión siguiente como borrador (la publicada sigue
  visible hasta publicar la nueva);
- fila con id y «sí» en retirar: se retiran todas sus versiones vigentes;
- sin cambios: nada. Quitar una fila no retira la pregunta.

Todo o nada, con errores por fila (un id desconocido también es error). La
plantilla antigua sigue sirviendo: id, estado y retirar son opcionales.
Retirar procede ahora desde cualquier estado y queda en content_event.

AC-044, modelo de dominio y docs/correcciones.md §W actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plantillas/preguntas-alternativas.xlsx
+++ b/docs/plantillas/preguntas-alternativas.xlsx
@@ -28,7 +28,6 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
     <font>
       <b val="1"/>
@@ -44,7 +43,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5BD3"/>
+        <fgColor rgb="00E8EEF9"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,14 +59,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,205 +428,223 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>materia</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>subtema</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>dificultad</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>enunciado</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>alternativa_a</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>alternativa_b</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>alternativa_c</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>alternativa_d</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>alternativa_e</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>correcta</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>explicacion</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>fuente</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>retirar</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Derecho Civil</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Personas</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>¿Cuándo principia la existencia legal de una persona?</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Desde la concepción</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Al nacer, esto es, al separarse completamente de su madre</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Al inscribirse en el Registro Civil</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>A las 24 horas de nacida</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>La existencia legal principia al nacimiento, al separarse completamente de la madre.</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Código Civil, art. 74</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Derecho Constitucional</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Presidente de la República</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="D3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>¿Cuánto dura el mandato del Presidente de la República?</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>4 años, sin reelección para el período siguiente</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>4 años, con reelección inmediata</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>6 años, sin reelección</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>5 años, con una reelección</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>El Presidente dura cuatro años y no puede ser reelegido para el período siguiente.</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Constitución Política de la República, art. 25</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Dificultad" error="La dificultad va de 1 a 3" type="whole" operator="between">
-      <formula1>1</formula1>
-      <formula2>3</formula2>
+  <dataValidations count="3">
+    <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elige una dificultad de la lista." type="list">
+      <formula1>"1,2,3"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Correcta" error="Escribe la letra de la alternativa correcta (A–E)" type="list">
+    <dataValidation sqref="K2:K5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Escribe la letra de la correcta (A–E)." type="list">
       <formula1>"A,B,C,D,E"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Escribe «sí» para retirar la pregunta, o déjalo vacío." type="list">
+      <formula1>"sí"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -645,102 +657,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Plantilla de preguntas — Aprueba tu examen</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Banco de preguntas — Aprueba tu examen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Una fila por pregunta en la hoja «Preguntas». Borra las 2 filas de ejemplo antes de enviar.</t>
+          <t>Una fila por pregunta, en la hoja «Preguntas». Al subir la planilla en /admin/preguntas:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>• Fila sin id → pregunta nueva, como borrador.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>materia: nombre de la materia (ej.: Derecho Civil).</t>
+          <t>• Fila con id y algún cambio → nueva versión de esa pregunta, como borrador. La versión anterior no se modifica y sigue publicada hasta que se publique la nueva.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>subtema: subtema dentro de la materia (cada materia puede tener los suyos).</t>
+          <t>• Fila con id y «sí» en la columna retirar → la pregunta se retira (deja de aparecer en la práctica). No se borra: queda en el historial.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dificultad: 1 = fácil, 2 = media, 3 = difícil (escala propuesta, por confirmar).</t>
+          <t>• Fila con id sin cambios → no pasa nada.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>enunciado: la pregunta, tal como la verá el estudiante.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>alternativa_a … alternativa_e: entre 2 y 5 alternativas; deja vacías las que no uses.</t>
-        </is>
-      </c>
-    </row>
+          <t>Borrar una fila de la planilla NO retira la pregunta: para sacarla, usa la columna retirar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>correcta: la letra de la alternativa correcta (A–E). Debe apuntar a una alternativa con texto.</t>
+          <t>No modifiques la columna id. La columna estado es solo informativa.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>explicacion: por qué es la correcta; se muestra al estudiante cuando se equivoca.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>fuente: artículo o norma que respalda la respuesta (ej.: Código Civil, art. 74).</t>
-        </is>
-      </c>
-    </row>
+          <t>Si alguna fila tiene un error, no se aplica ningún cambio y se informa cada fila.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Columnas:</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Nada se publica directamente: al importar, cada pregunta queda como borrador para revisión.</t>
+          <t>materia: nombre de la materia (ej.: Derecho Civil).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Quien crea o modifica una pregunta no puede aprobarla ni publicarla (otra persona la revisa).</t>
+          <t>subtema: subtema dentro de la materia (opcional).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>dificultad: 1 = fácil, 2 = media, 3 = difícil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>enunciado: la pregunta, tal como la verá el estudiante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>alternativa_a … alternativa_e: entre 2 y 5 alternativas, seguidas y sin repetir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>correcta: la letra de la alternativa correcta (A, B, C, D o E).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>explicacion: por qué la correcta es correcta (y, idealmente, por qué las demás no).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>fuente: artículo, ley o texto de respaldo (hasta 300 caracteres).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Toda pregunta nueva o modificada debe revisarla y publicarla otro administrador.</t>
         </is>
       </c>
     </row>

</xml_diff>